<commit_message>
Add product reviews dataset with 100 entries across various categories
</commit_message>
<xml_diff>
--- a/static/outputs/lumiq_report.xlsx
+++ b/static/outputs/lumiq_report.xlsx
@@ -6573,7 +6573,7 @@
         </is>
       </c>
       <c r="G14" s="15" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="15">
@@ -6608,7 +6608,7 @@
         </is>
       </c>
       <c r="G15" s="15" t="n">
-        <v>0.46</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="16">
@@ -6643,7 +6643,7 @@
         </is>
       </c>
       <c r="G16" s="19" t="n">
-        <v>0.61</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="17">
@@ -6678,7 +6678,7 @@
         </is>
       </c>
       <c r="G17" s="15" t="n">
-        <v>0.7</v>
+        <v>0.35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add comprehensive results dashboard with integrated data visualization, sentiment analysis, and reporting tools
</commit_message>
<xml_diff>
--- a/static/outputs/lumiq_report.xlsx
+++ b/static/outputs/lumiq_report.xlsx
@@ -6573,7 +6573,7 @@
         </is>
       </c>
       <c r="G14" s="15" t="n">
-        <v>0.41</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="15">
@@ -6608,7 +6608,7 @@
         </is>
       </c>
       <c r="G15" s="15" t="n">
-        <v>0.31</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="16">
@@ -6643,7 +6643,7 @@
         </is>
       </c>
       <c r="G16" s="19" t="n">
-        <v>0.36</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="17">
@@ -6678,7 +6678,7 @@
         </is>
       </c>
       <c r="G17" s="15" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add project data infrastructure and update file copying logic in app.py
</commit_message>
<xml_diff>
--- a/static/outputs/lumiq_report.xlsx
+++ b/static/outputs/lumiq_report.xlsx
@@ -6610,7 +6610,7 @@
         </is>
       </c>
       <c r="G15" s="15" t="n">
-        <v>0.4</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="16">
@@ -6645,7 +6645,7 @@
         </is>
       </c>
       <c r="G16" s="19" t="n">
-        <v>0.26</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="17">
@@ -6680,7 +6680,7 @@
         </is>
       </c>
       <c r="G17" s="15" t="n">
-        <v>0.17</v>
+        <v>0.29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
some UI and other changes
</commit_message>
<xml_diff>
--- a/static/outputs/lumiq_report.xlsx
+++ b/static/outputs/lumiq_report.xlsx
@@ -6610,7 +6610,7 @@
         </is>
       </c>
       <c r="G15" s="15" t="n">
-        <v>0.52</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="16">
@@ -6645,7 +6645,7 @@
         </is>
       </c>
       <c r="G16" s="19" t="n">
-        <v>0.31</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="17">
@@ -6680,7 +6680,7 @@
         </is>
       </c>
       <c r="G17" s="15" t="n">
-        <v>0.29</v>
+        <v>0.24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>